<commit_message>
small changes in code
</commit_message>
<xml_diff>
--- a/appointments_summary.xlsx
+++ b/appointments_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,17 +441,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>date</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>time</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -471,32 +471,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>xyz</t>
+          <t>souj</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cold cough</t>
+          <t>9872737461</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>headache</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>General Medicine</t>
+          <t>Accident &amp; Emergency</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Auto-assigned</t>
+          <t>Dr. Aruna C Ramesh</t>
         </is>
       </c>
     </row>
@@ -506,32 +506,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>dee</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chest pain</t>
+          <t>9483869206</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2023-10-12</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Endocrinology</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dr. Smith</t>
+          <t>Dr. Pramila Kalra</t>
         </is>
       </c>
     </row>
@@ -541,32 +541,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>abbu</t>
+          <t>dee</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>backpain</t>
+          <t>8088091773</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>General Medicine</t>
+          <t>Critical Care Medicine</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>john</t>
+          <t>Dr. Deepak T S</t>
         </is>
       </c>
     </row>
@@ -576,32 +576,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Test Patient</t>
+          <t>deeksha</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chest pain</t>
+          <t>8088091773</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>leg pain</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Accident &amp; Emergency</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dr. Test</t>
+          <t>Dr. Aruna C Ramesh</t>
         </is>
       </c>
     </row>
@@ -611,242 +611,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>chi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>headache</t>
+          <t>9483869206</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-05-05</t>
+          <t>body pain</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>neurology</t>
+          <t>General Medicine</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Auto-assigned</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>DEE</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>leg pain</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>General Medicine</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Liam</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Difficulty breathing</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2023-10-25</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Emergency</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Auto-assigned</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Akash</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>headache</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>neurology</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Auto-assigned</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Shah</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>stomachache</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>gastroenterology</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Auto-assigned</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>gana</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>heart</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Cardiology</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Dr. Arjun Dev</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>chaii</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>leg injury</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>General Medicine</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Dr. Sanjay Gupta</t>
+          <t>Dr. Shaikh Mohammed Aslam S</t>
         </is>
       </c>
     </row>

</xml_diff>